<commit_message>
Rewrite the data file pipeline
</commit_message>
<xml_diff>
--- a/data/raw/rules.xlsx
+++ b/data/raw/rules.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="140">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -31,7 +31,10 @@
     <t xml:space="preserve">type</t>
   </si>
   <si>
-    <t xml:space="preserve">source</t>
+    <t xml:space="preserve">source_book</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source_page</t>
   </si>
   <si>
     <t xml:space="preserve">heroic-accuracy</t>
@@ -43,7 +46,7 @@
     <t xml:space="preserve">shoot-phase</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 83)</t>
+    <t xml:space="preserve">rules-manual</t>
   </si>
   <si>
     <t xml:space="preserve">heroic-challenge</t>
@@ -52,39 +55,24 @@
     <t xml:space="preserve">fight-phase</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 82)</t>
-  </si>
-  <si>
     <t xml:space="preserve">heroic-channelling</t>
   </si>
   <si>
     <t xml:space="preserve">move-phase</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 84)</t>
-  </si>
-  <si>
     <t xml:space="preserve">heroic-combat</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 81)</t>
-  </si>
-  <si>
     <t xml:space="preserve">heroic-defence</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 85)</t>
-  </si>
-  <si>
     <t xml:space="preserve">heroic-march</t>
   </si>
   <si>
     <t xml:space="preserve">heroic-move</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 80)</t>
-  </si>
-  <si>
     <t xml:space="preserve">heroic-resolve</t>
   </si>
   <si>
@@ -106,9 +94,6 @@
     <t xml:space="preserve">exhaustion</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 116)</t>
-  </si>
-  <si>
     <t xml:space="preserve">aura-of-dismay</t>
   </si>
   <si>
@@ -139,9 +124,6 @@
     <t xml:space="preserve">chill-soul</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 117)</t>
-  </si>
-  <si>
     <t xml:space="preserve">collapse-rocks</t>
   </si>
   <si>
@@ -166,9 +148,6 @@
     <t xml:space="preserve">fog-of-disarray</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 118)</t>
-  </si>
-  <si>
     <t xml:space="preserve">foil-magic</t>
   </si>
   <si>
@@ -193,9 +172,6 @@
     <t xml:space="preserve">protection-of-the-valar</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 119)</t>
-  </si>
-  <si>
     <t xml:space="preserve">renew</t>
   </si>
   <si>
@@ -217,9 +193,6 @@
     <t xml:space="preserve">wither</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 120)</t>
-  </si>
-  <si>
     <t xml:space="preserve">wrath-of-bruinen</t>
   </si>
   <si>
@@ -238,9 +211,6 @@
     <t xml:space="preserve">active</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 124)</t>
-  </si>
-  <si>
     <t xml:space="preserve">backstabbers</t>
   </si>
   <si>
@@ -265,9 +235,6 @@
     <t xml:space="preserve">cave-dweller</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 125)</t>
-  </si>
-  <si>
     <t xml:space="preserve">dominant</t>
   </si>
   <si>
@@ -289,9 +256,6 @@
     <t xml:space="preserve">fly</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 126)</t>
-  </si>
-  <si>
     <t xml:space="preserve">general-hunter</t>
   </si>
   <si>
@@ -304,9 +268,6 @@
     <t xml:space="preserve">horse-lord</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 127)</t>
-  </si>
-  <si>
     <t xml:space="preserve">invisible</t>
   </si>
   <si>
@@ -325,9 +286,6 @@
     <t xml:space="preserve">mighty-hero</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 128)</t>
-  </si>
-  <si>
     <t xml:space="preserve">monstrous-charge</t>
   </si>
   <si>
@@ -346,9 +304,6 @@
     <t xml:space="preserve">sharpshooter</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 129)</t>
-  </si>
-  <si>
     <t xml:space="preserve">shieldwall</t>
   </si>
   <si>
@@ -367,9 +322,6 @@
     <t xml:space="preserve">sworn-protector</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 130)</t>
-  </si>
-  <si>
     <t xml:space="preserve">terror</t>
   </si>
   <si>
@@ -385,9 +337,6 @@
     <t xml:space="preserve">venom</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 131)</t>
-  </si>
-  <si>
     <t xml:space="preserve">will-of-evil</t>
   </si>
   <si>
@@ -400,27 +349,18 @@
     <t xml:space="preserve">brutal-power-attack</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 90)</t>
-  </si>
-  <si>
     <t xml:space="preserve">rend</t>
   </si>
   <si>
     <t xml:space="preserve">hurl</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 91)</t>
-  </si>
-  <si>
     <t xml:space="preserve">hand-weapon</t>
   </si>
   <si>
     <t xml:space="preserve">equipment</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 103)</t>
-  </si>
-  <si>
     <t xml:space="preserve">two-handed-weapon</t>
   </si>
   <si>
@@ -433,18 +373,12 @@
     <t xml:space="preserve">spear</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 104)</t>
-  </si>
-  <si>
     <t xml:space="preserve">pike</t>
   </si>
   <si>
     <t xml:space="preserve">lance</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 105)</t>
-  </si>
-  <si>
     <t xml:space="preserve">war-spear</t>
   </si>
   <si>
@@ -463,9 +397,6 @@
     <t xml:space="preserve">bow</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 106)</t>
-  </si>
-  <si>
     <t xml:space="preserve">throwing-weapon</t>
   </si>
   <si>
@@ -481,15 +412,9 @@
     <t xml:space="preserve">banner</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 107)</t>
-  </si>
-  <si>
     <t xml:space="preserve">elven-cloak</t>
   </si>
   <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 108)</t>
-  </si>
-  <si>
     <t xml:space="preserve">war-drum</t>
   </si>
   <si>
@@ -497,9 +422,6 @@
   </si>
   <si>
     <t xml:space="preserve">armour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 109)</t>
   </si>
   <si>
     <t xml:space="preserve">light-armour</t>
@@ -527,7 +449,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -549,6 +471,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -593,7 +521,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -608,6 +536,14 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -627,13 +563,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D123"/>
-  <sheetFormatPr defaultColWidth="8.5234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E123"/>
+  <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="53.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -649,33 +586,42 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
         <v>7</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
         <v>10</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -683,1572 +629,1929 @@
         <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>81</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>10</v>
+      <c r="D7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>20</v>
+      <c r="D8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>7</v>
+      <c r="D9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>15</v>
+        <v>7</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>81</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>28</v>
+      <c r="D15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>28</v>
+      <c r="D16" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>28</v>
+      <c r="D18" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>28</v>
+      <c r="D20" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>39</v>
+      <c r="D21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>39</v>
+      <c r="D22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>39</v>
+      <c r="D23" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>39</v>
+      <c r="D24" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>39</v>
+      <c r="D25" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>39</v>
+        <v>29</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>39</v>
+        <v>29</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>39</v>
+      <c r="D28" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>48</v>
+        <v>23</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>48</v>
+      <c r="D30" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>48</v>
+        <v>23</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>48</v>
+        <v>23</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>48</v>
+        <v>29</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>48</v>
+      <c r="D34" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C35" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>48</v>
+      <c r="D35" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>48</v>
+        <v>23</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>57</v>
+        <v>29</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>57</v>
+      <c r="D38" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C39" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>57</v>
+      <c r="D39" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>57</v>
+      <c r="D40" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>57</v>
+        <v>23</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>57</v>
+        <v>29</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C43" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>57</v>
+      <c r="D43" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>119</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C44" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>65</v>
+      <c r="D44" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C45" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>65</v>
+      <c r="D45" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>65</v>
+        <v>29</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="B47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C47" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>65</v>
+      <c r="D47" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>72</v>
+        <v>62</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>72</v>
+        <v>62</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>72</v>
+        <v>62</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>72</v>
+        <v>62</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>72</v>
+        <v>62</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" s="5" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>124</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>81</v>
+        <v>62</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" s="5" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>81</v>
+        <v>68</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" s="5" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>81</v>
+        <v>62</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" s="5" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>81</v>
+        <v>62</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>81</v>
+        <v>68</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" s="5" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>81</v>
+        <v>68</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>81</v>
+        <v>68</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" s="5" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>89</v>
+        <v>62</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62" s="5" t="n">
+        <v>126</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>89</v>
+        <v>62</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63" s="5" t="n">
+        <v>126</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>89</v>
+        <v>68</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" s="5" t="n">
+        <v>126</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>89</v>
+        <v>62</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" s="5" t="n">
+        <v>126</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66" s="5" t="n">
+        <v>127</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67" s="5" t="n">
+        <v>127</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E68" s="5" t="n">
+        <v>127</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E69" s="5" t="n">
+        <v>127</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>94</v>
+        <v>62</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E70" s="5" t="n">
+        <v>127</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>94</v>
+        <v>62</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" s="5" t="n">
+        <v>127</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>101</v>
+        <v>68</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72" s="5" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>101</v>
+        <v>62</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E73" s="5" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>101</v>
+        <v>62</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E74" s="5" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>101</v>
+        <v>62</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E75" s="5" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>101</v>
+        <v>68</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E76" s="5" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>101</v>
+        <v>68</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E77" s="5" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>108</v>
+        <v>62</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E78" s="5" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>108</v>
+        <v>62</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E79" s="5" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>108</v>
+        <v>68</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E80" s="5" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>108</v>
+        <v>68</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E81" s="5" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>108</v>
+        <v>62</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E82" s="5" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>108</v>
+        <v>62</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E83" s="5" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>115</v>
+        <v>68</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E84" s="5" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>115</v>
+        <v>68</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E85" s="5" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>115</v>
+        <v>62</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E86" s="5" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>115</v>
+        <v>68</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E87" s="5" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>115</v>
+        <v>62</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E88" s="5" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>121</v>
+        <v>62</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E89" s="5" t="n">
+        <v>131</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>121</v>
+        <v>68</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E90" s="5" t="n">
+        <v>131</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>121</v>
+        <v>62</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E91" s="5" t="n">
+        <v>131</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>126</v>
+        <v>108</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E92" s="5" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>126</v>
+        <v>108</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E93" s="5" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>129</v>
+        <v>108</v>
+      </c>
+      <c r="D94" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E94" s="5" t="n">
+        <v>91</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>132</v>
+        <v>112</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E95" s="5" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="0" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>132</v>
+        <v>112</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E96" s="5" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="0" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D97" s="2" t="s">
-        <v>132</v>
+        <v>112</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97" s="5" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>132</v>
+        <v>112</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E98" s="5" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="0" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>137</v>
+        <v>112</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E99" s="5" t="n">
+        <v>104</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="0" t="s">
-        <v>138</v>
+        <v>117</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D100" s="2" t="s">
-        <v>137</v>
+        <v>112</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E100" s="5" t="n">
+        <v>104</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="0" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D101" s="2" t="s">
-        <v>140</v>
+        <v>112</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E101" s="5" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="0" t="s">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>140</v>
+        <v>112</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E102" s="5" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="0" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>140</v>
+        <v>112</v>
+      </c>
+      <c r="D103" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E103" s="5" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="0" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>140</v>
+        <v>112</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E104" s="5" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="0" t="s">
-        <v>144</v>
+        <v>122</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D105" s="2" t="s">
-        <v>140</v>
+        <v>112</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E105" s="5" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="0" t="s">
-        <v>145</v>
+        <v>123</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>140</v>
+        <v>112</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E106" s="5" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="0" t="s">
-        <v>146</v>
+        <v>124</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>147</v>
+        <v>112</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E107" s="5" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="0" t="s">
-        <v>148</v>
+        <v>125</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D108" s="2" t="s">
-        <v>147</v>
+        <v>112</v>
+      </c>
+      <c r="D108" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E108" s="5" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="0" t="s">
-        <v>149</v>
+        <v>126</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>147</v>
+        <v>112</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E109" s="5" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="0" t="s">
-        <v>150</v>
+        <v>127</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>147</v>
+        <v>112</v>
+      </c>
+      <c r="D110" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E110" s="5" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="0" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>147</v>
+        <v>112</v>
+      </c>
+      <c r="D111" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E111" s="5" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="0" t="s">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D112" s="2" t="s">
-        <v>153</v>
+        <v>112</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E112" s="5" t="n">
+        <v>107</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="0" t="s">
-        <v>154</v>
+        <v>130</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>155</v>
+        <v>112</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E113" s="5" t="n">
+        <v>108</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="0" t="s">
-        <v>156</v>
+        <v>131</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D114" s="2" t="s">
-        <v>155</v>
+        <v>112</v>
+      </c>
+      <c r="D114" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E114" s="5" t="n">
+        <v>108</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="0" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>155</v>
+        <v>112</v>
+      </c>
+      <c r="D115" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E115" s="5" t="n">
+        <v>108</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="0" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D116" s="2" t="s">
-        <v>159</v>
+        <v>112</v>
+      </c>
+      <c r="D116" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E116" s="5" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="0" t="s">
-        <v>160</v>
+        <v>134</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D117" s="2" t="s">
-        <v>159</v>
+        <v>112</v>
+      </c>
+      <c r="D117" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E117" s="5" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="0" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>159</v>
+        <v>112</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E118" s="5" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="0" t="s">
-        <v>162</v>
+        <v>136</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>159</v>
+        <v>112</v>
+      </c>
+      <c r="D119" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E119" s="5" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="0" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D120" s="2" t="s">
-        <v>159</v>
+        <v>112</v>
+      </c>
+      <c r="D120" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E120" s="5" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="0" t="s">
-        <v>164</v>
+        <v>138</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D121" s="2" t="s">
-        <v>159</v>
+        <v>112</v>
+      </c>
+      <c r="D121" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E121" s="5" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="0" t="s">
-        <v>165</v>
+        <v>139</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>159</v>
+        <v>112</v>
+      </c>
+      <c r="D122" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E122" s="5" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>